<commit_message>
Fix SQLite detection on broad directory searches
</commit_message>
<xml_diff>
--- a/fixtures/sample.xlsx
+++ b/fixtures/sample.xlsx
@@ -1,9 +1,17 @@
+
+<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheets>
+    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+  </sheets>
+</workbook>
+</file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetData>
-    <row>
-      <c t="inlineStr">
+    <row r="1">
+      <c r="A1" t="inlineStr">
         <is>
           <t>NEEDLE_7429 xlsx</t>
         </is>

</xml_diff>